<commit_message>
build_one_file_rosetta: reverse complement strand-flipped single-base C/T long_visual
So every occurrence of a single-base C/T class can serve as an example and
no (476-type, 89-type) block is left without an indel in context.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CXqMg6LHHkTRCFtEjwRvwQ
</commit_message>
<xml_diff>
--- a/development/one_file_rosetta_output/SP112959_rosetta.xlsx
+++ b/development/one_file_rosetta_output/SP112959_rosetta.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="17.711"/>
@@ -4282,7 +4282,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TCTGA</t>
+            <t>AGAAA</t>
           </r>
           <r>
             <rPr>
@@ -4308,7 +4308,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AAAGCCAGAAAATAAGGGAA</t>
+            <t>AAAACTAATCCTTAGTGACT</t>
           </r>
         </is>
       </c>
@@ -4316,24 +4316,24 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>Del(10,):U1:R1</t>
+          <t>A[Del(C):R1]A</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t>Del(5,):R1</t>
+          <t>[Del(C):R1]A</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>DEL:repeats:5+:0</t>
+          <t>DEL:C:1:0</t>
         </is>
       </c>
       <c r="D37" s="4">
         <v>2</v>
       </c>
       <c r="E37" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
@@ -4341,7 +4341,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TTTTG</t>
+            <t>TCTGA</t>
           </r>
           <r>
             <rPr>
@@ -4355,7 +4355,7 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AAAACTTTTTTCT</t>
+            <t>C</t>
           </r>
           <r>
             <rPr>
@@ -4367,7 +4367,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TCCCAGTACGTAGAGAAATC</t>
+            <t>AAAGCCAGAAAATAAGGGAA</t>
           </r>
         </is>
       </c>
@@ -4392,7 +4392,7 @@
         <v>2</v>
       </c>
       <c r="E38" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
@@ -4400,7 +4400,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TTTTT</t>
+            <t>TTTTG</t>
           </r>
           <r>
             <rPr>
@@ -4414,7 +4414,7 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>CCTTTCAAAG</t>
+            <t>AAAACTTTTTTCT</t>
           </r>
           <r>
             <rPr>
@@ -4426,7 +4426,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AATATGCTTCCTACATGCTG</t>
+            <t>TCCCAGTACGTAGAGAAATC</t>
           </r>
         </is>
       </c>
@@ -4434,24 +4434,24 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>Del3:M2</t>
+          <t>Del(10,):U1:R1</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>Del(3,5):M2</t>
+          <t>Del(5,):R1</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>DEL:MH:3:2</t>
+          <t>DEL:repeats:5+:0</t>
         </is>
       </c>
       <c r="D39" s="4">
         <v>2</v>
       </c>
       <c r="E39" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
@@ -4459,7 +4459,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>ATTTC</t>
+            <t>TTTTT</t>
           </r>
           <r>
             <rPr>
@@ -4470,19 +4470,10 @@
           <r>
             <rPr>
               <b/>
-              <u val="double"/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AC</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>G</t>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CCTTTCAAAG</t>
           </r>
           <r>
             <rPr>
@@ -4492,16 +4483,9 @@
           </r>
           <r>
             <rPr>
-              <u val="double"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AC</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AAGTATCAAAACTGTCCACT</t>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AATATGCTTCCTACATGCTG</t>
           </r>
         </is>
       </c>
@@ -4526,7 +4510,7 @@
         <v>2</v>
       </c>
       <c r="E40" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
@@ -4534,7 +4518,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TCCTC</t>
+            <t>ATTTC</t>
           </r>
           <r>
             <rPr>
@@ -4549,15 +4533,15 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>CT</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>T</t>
+            <t>AC</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>G</t>
           </r>
           <r>
             <rPr>
@@ -4570,13 +4554,13 @@
               <u val="double"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>CT</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AGTTCATTAATTGATCTTGG</t>
+            <t>AC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AAGTATCAAAACTGTCCACT</t>
           </r>
         </is>
       </c>
@@ -4584,30 +4568,74 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>A[Del(C):R2]T</t>
+          <t>Del3:M2</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
-          <t>[Del(C):R2]T</t>
+          <t>Del(3,5):M2</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t/>
+          <t>DEL:MH:3:2</t>
         </is>
       </c>
       <c r="D41" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E41" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
           <r>
-            <rPr/>
-            <t/>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>TCCTC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <u val="double"/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CT</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <u val="double"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AGTTCATTAATTGATCTTGG</t>
           </r>
         </is>
       </c>
@@ -4615,17 +4643,17 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>T[Del(C):R3]A</t>
+          <t>A[Del(C):R2]T</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
-          <t>[Del(C):R3]A</t>
+          <t>[Del(C):R2]T</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>DEL:C:1:2</t>
+          <t>DEL:C:1:1</t>
         </is>
       </c>
       <c r="D42" s="4">
@@ -4640,7 +4668,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GTTCT</t>
+            <t>CAAAA</t>
           </r>
           <r>
             <rPr>
@@ -4671,17 +4699,9 @@
           </r>
           <r>
             <rPr>
-              <u/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>C</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AAAATTCAGTACTTCTGGC</t>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>TTTTTACCTATAATAACAAA</t>
           </r>
         </is>
       </c>
@@ -4689,17 +4709,17 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>A[Del(T):R2]C</t>
+          <t>T[Del(C):R3]A</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
-          <t>A[Del(T):R(1,4)]C</t>
+          <t>[Del(C):R3]A</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>DEL:T:1:1</t>
+          <t>DEL:C:1:2</t>
         </is>
       </c>
       <c r="D43" s="4">
@@ -4714,7 +4734,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TATGA</t>
+            <t>GTTCT</t>
           </r>
           <r>
             <rPr>
@@ -4728,7 +4748,7 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>T</t>
+            <t>C</t>
           </r>
           <r>
             <rPr>
@@ -4741,13 +4761,21 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>T</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>CTACACCTAGAAAACCCCAT</t>
+            <t>C</t>
+          </r>
+          <r>
+            <rPr>
+              <u/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>C</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AAAATTCAGTACTTCTGGC</t>
           </r>
         </is>
       </c>
@@ -4755,17 +4783,17 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>A[Del(T):R4]G</t>
+          <t>A[Del(T):R2]C</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
-          <t>A[Del(T):R(1,4)]G</t>
+          <t>A[Del(T):R(1,4)]C</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t/>
+          <t>DEL:T:1:1</t>
         </is>
       </c>
       <c r="D44" s="4">
@@ -4777,8 +4805,43 @@
       <c r="F44" s="6" t="inlineStr">
         <is>
           <r>
-            <rPr/>
-            <t/>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>TATGA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CTACACCTAGAAAACCCCAT</t>
           </r>
         </is>
       </c>
@@ -4786,17 +4849,17 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>A[Del(T):R5]A</t>
+          <t>A[Del(T):R4]G</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t>A[Del(T):R(5,7)]A</t>
+          <t>A[Del(T):R(1,4)]G</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>DEL:T:1:4</t>
+          <t>DEL:T:1:3</t>
         </is>
       </c>
       <c r="D45" s="4">
@@ -4811,7 +4874,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>ATTTA</t>
+            <t>TCCCA</t>
           </r>
           <r>
             <rPr>
@@ -4857,17 +4920,9 @@
           </r>
           <r>
             <rPr>
-              <u/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>T</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AGAGGTAAAAAATTCTT</t>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GTATGTTGCCTGTTCACTCT</t>
           </r>
         </is>
       </c>
@@ -4875,17 +4930,17 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>C[Del(T):R3]C</t>
+          <t>A[Del(T):R5]A</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>C[Del(T):R(1,4)]C</t>
+          <t>A[Del(T):R(5,7)]A</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t/>
+          <t>DEL:T:1:4</t>
         </is>
       </c>
       <c r="D46" s="4">
@@ -4897,8 +4952,66 @@
       <c r="F46" s="6" t="inlineStr">
         <is>
           <r>
-            <rPr/>
-            <t/>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>ATTTA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <u/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <u/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AGAGGTAAAAAATTCTT</t>
           </r>
         </is>
       </c>
@@ -4906,17 +5019,17 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>G[Del(T):R2]A</t>
+          <t>C[Del(T):R3]C</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
-          <t>G[Del(T):R(1,4)]A</t>
+          <t>C[Del(T):R(1,4)]C</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>DEL:T:1:1</t>
+          <t>DEL:T:1:2</t>
         </is>
       </c>
       <c r="D47" s="4">
@@ -4931,7 +5044,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>CACAG</t>
+            <t>CGTTC</t>
           </r>
           <r>
             <rPr>
@@ -4962,9 +5075,17 @@
           </r>
           <r>
             <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AGGACAGGCTATTGGGGTTC</t>
+              <u/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CTATATTTGTGCTGAATCTA</t>
           </r>
         </is>
       </c>
@@ -4972,17 +5093,17 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>G[Del(T):R2]C</t>
+          <t>G[Del(T):R2]A</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
-          <t>G[Del(T):R(1,4)]C</t>
+          <t>G[Del(T):R(1,4)]A</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t/>
+          <t>DEL:T:1:1</t>
         </is>
       </c>
       <c r="D48" s="4">
@@ -4994,8 +5115,43 @@
       <c r="F48" s="6" t="inlineStr">
         <is>
           <r>
-            <rPr/>
-            <t/>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CACAG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AGGACAGGCTATTGGGGTTC</t>
           </r>
         </is>
       </c>
@@ -5003,17 +5159,17 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>A[Ins(T):R(9,)]C</t>
+          <t>G[Del(T):R2]C</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
-          <t>A[Ins(T):R(8,)]C</t>
+          <t>G[Del(T):R(1,4)]C</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>INS:T:1:5+</t>
+          <t>DEL:T:1:1</t>
         </is>
       </c>
       <c r="D49" s="4">
@@ -5028,7 +5184,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TTTTA</t>
+            <t>TGCTG</t>
           </r>
           <r>
             <rPr>
@@ -5059,69 +5215,9 @@
           </r>
           <r>
             <rPr>
-              <u/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>T</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>T</t>
-          </r>
-          <r>
-            <rPr>
-              <u/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>T</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>T</t>
-          </r>
-          <r>
-            <rPr>
-              <u/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>T</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>T</t>
-          </r>
-          <r>
-            <rPr>
-              <u/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>T</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>T</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>CTTGCCTAACTG</t>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CCACTTGTTCCTAAATCCCT</t>
           </r>
         </is>
       </c>
@@ -5129,12 +5225,12 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>C[Ins(T):R(9,)]G</t>
+          <t>A[Ins(T):R(9,)]C</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
-          <t>C[Ins(T):R(8,)]G</t>
+          <t>A[Ins(T):R(8,)]C</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
@@ -5154,7 +5250,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TTGGC</t>
+            <t>TTTTA</t>
           </r>
           <r>
             <rPr>
@@ -5247,7 +5343,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GGAGACGGAGTT</t>
+            <t>CTTGCCTAACTG</t>
           </r>
         </is>
       </c>
@@ -5255,17 +5351,17 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>Del2:U2:R2</t>
+          <t>C[Ins(T):R(9,)]G</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
-          <t>Del(2,8):U(1,2):R(2,4)</t>
+          <t>C[Ins(T):R(8,)]G</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>DEL:repeats:2:1</t>
+          <t>INS:T:1:5+</t>
         </is>
       </c>
       <c r="D51" s="4">
@@ -5280,7 +5376,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TGTAA</t>
+            <t>TTGGC</t>
           </r>
           <r>
             <rPr>
@@ -5294,7 +5390,7 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AC</t>
+            <t>T</t>
           </r>
           <r>
             <rPr>
@@ -5307,13 +5403,73 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AC</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AGTCAAAAGAGATTAAGTAT</t>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <u/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <u/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <u/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <u/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GGAGACGGAGTT</t>
           </r>
         </is>
       </c>
@@ -5321,17 +5477,17 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>Del3:U3:R3</t>
+          <t>Del2:U2:R2</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
-          <t>Del(3,):U(3,):R(3,)</t>
+          <t>Del(2,8):U(1,2):R(2,4)</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>DEL:repeats:3:2</t>
+          <t>DEL:repeats:2:1</t>
         </is>
       </c>
       <c r="D52" s="4">
@@ -5346,7 +5502,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AGGAG</t>
+            <t>TGTAA</t>
           </r>
           <r>
             <rPr>
@@ -5360,7 +5516,7 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>ACC</t>
+            <t>AC</t>
           </r>
           <r>
             <rPr>
@@ -5373,21 +5529,13 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>ACC</t>
-          </r>
-          <r>
-            <rPr>
-              <u/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>ACC</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>ACTTTCACTCTAAATTAGCA</t>
+            <t>AC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AGTCAAAAGAGATTAAGTAT</t>
           </r>
         </is>
       </c>
@@ -5395,17 +5543,17 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>Ins4:U2:R2</t>
+          <t>Del3:U3:R3</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
-          <t>Ins(2,):R(2,4)</t>
+          <t>Del(3,):U(3,):R(3,)</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>INS:repeats:4:1</t>
+          <t>DEL:repeats:3:2</t>
         </is>
       </c>
       <c r="D53" s="4">
@@ -5420,7 +5568,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>ATGAT</t>
+            <t>AGGAG</t>
           </r>
           <r>
             <rPr>
@@ -5434,7 +5582,7 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TATA</t>
+            <t>ACC</t>
           </r>
           <r>
             <rPr>
@@ -5447,13 +5595,21 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TATA</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>CCACTGTACTCCAGCAGGGG</t>
+            <t>ACC</t>
+          </r>
+          <r>
+            <rPr>
+              <u/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>ACC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>ACTTTCACTCTAAATTAGCA</t>
           </r>
         </is>
       </c>
@@ -5461,17 +5617,17 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>Ins(5,):U(3,):R(5,)</t>
+          <t>Ins4:U2:R2</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
-          <t>Ins(2,):R(5,)</t>
+          <t>Ins(2,):R(2,4)</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>INS:repeats:5+:5+</t>
+          <t>INS:repeats:4:1</t>
         </is>
       </c>
       <c r="D54" s="4">
@@ -5486,7 +5642,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AGAAG</t>
+            <t>ATGAT</t>
           </r>
           <r>
             <rPr>
@@ -5500,7 +5656,7 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GAAAGAAA</t>
+            <t>TATA</t>
           </r>
           <r>
             <rPr>
@@ -5513,51 +5669,13 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GAAAGAAA</t>
-          </r>
-          <r>
-            <rPr>
-              <u/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GAAAGAAA</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GAAAGAAA</t>
-          </r>
-          <r>
-            <rPr>
-              <u/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GAAAGAAA</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GAAAGAAA</t>
-          </r>
-          <r>
-            <rPr>
-              <u/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GAAAGAAA</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GAAAAGAAAGAAAGAAAGAG</t>
+            <t>TATA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CCACTGTACTCCAGCAGGGG</t>
           </r>
         </is>
       </c>
@@ -5565,17 +5683,17 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>Del3:M1</t>
+          <t>Ins(5,):U(3,):R(5,)</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
-          <t>Del(2,5):M1</t>
+          <t>Ins(2,):R(5,)</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>DEL:MH:3:1</t>
+          <t>INS:repeats:5+:5+</t>
         </is>
       </c>
       <c r="D55" s="4">
@@ -5590,7 +5708,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TAGGT</t>
+            <t>AGAAG</t>
           </r>
           <r>
             <rPr>
@@ -5601,19 +5719,10 @@
           <r>
             <rPr>
               <b/>
-              <u val="double"/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>G</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GA</t>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GAAAGAAA</t>
           </r>
           <r>
             <rPr>
@@ -5623,16 +5732,54 @@
           </r>
           <r>
             <rPr>
-              <u val="double"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>G</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AAGTTTAAGTCAATGGATTA</t>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GAAAGAAA</t>
+          </r>
+          <r>
+            <rPr>
+              <u/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GAAAGAAA</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GAAAGAAA</t>
+          </r>
+          <r>
+            <rPr>
+              <u/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GAAAGAAA</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GAAAGAAA</t>
+          </r>
+          <r>
+            <rPr>
+              <u/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GAAAGAAA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GAAAAGAAAGAAAGAAAGAG</t>
           </r>
         </is>
       </c>
@@ -5640,7 +5787,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>Del4:M1</t>
+          <t>Del3:M1</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -5650,7 +5797,7 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>DEL:MH:4:1</t>
+          <t>DEL:MH:3:1</t>
         </is>
       </c>
       <c r="D56" s="4">
@@ -5665,7 +5812,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GTAAC</t>
+            <t>TAGGT</t>
           </r>
           <r>
             <rPr>
@@ -5680,15 +5827,15 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>T</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>ATT</t>
+            <t>G</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GA</t>
           </r>
           <r>
             <rPr>
@@ -5701,13 +5848,13 @@
               <u val="double"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>T</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GTTTGTTTTTCTGCTTCTAA</t>
+            <t>G</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AAGTTTAAGTCAATGGATTA</t>
           </r>
         </is>
       </c>
@@ -5715,17 +5862,17 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>Del(7,):M3</t>
+          <t>Del4:M1</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
-          <t>Del(6,):M3</t>
+          <t>Del(2,5):M1</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>DEL:MH:5+:3</t>
+          <t>DEL:MH:4:1</t>
         </is>
       </c>
       <c r="D57" s="4">
@@ -5740,6 +5887,81 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
+            <t>GTAAC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <u val="double"/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>ATT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <u val="double"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GTTTGTTTTTCTGCTTCTAA</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t>Del(7,):M3</t>
+        </is>
+      </c>
+      <c r="B58" s="1" t="inlineStr">
+        <is>
+          <t>Del(6,):M3</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>DEL:MH:5+:3</t>
+        </is>
+      </c>
+      <c r="D58" s="4">
+        <v>1</v>
+      </c>
+      <c r="E58" s="4">
+        <v>1</v>
+      </c>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
             <t>GACGG</t>
           </r>
           <r>
@@ -5788,7 +6010,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="24">
     <mergeCell ref="A2:A21"/>
     <mergeCell ref="B2:B21"/>
     <mergeCell ref="C2:C21"/>
@@ -5801,14 +6023,18 @@
     <mergeCell ref="B33:B35"/>
     <mergeCell ref="C33:C35"/>
     <mergeCell ref="D33:D35"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="D37:D38"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="D39:D40"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="D40:D41"/>
   </mergeCells>
   <printOptions gridLines="1" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>